<commit_message>
Automatisches Update TM + Transfers - 10.06.2025 10:24
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24DB1FB6-2729-445E-A16F-E01C93C29455}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39920400-FD7E-4F36-B782-1EA50BD09E83}"/>
   <bookViews>
-    <workbookView xWindow="5970" yWindow="5510" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
+    <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="146">
   <si>
     <t>Datum</t>
   </si>
@@ -456,6 +456,27 @@
   </si>
   <si>
     <t xml:space="preserve"> Widmer</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P. Nebel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Vagnoman</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Amiri</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Christoph</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Schmitz</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Juranovic</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> K. Müller</t>
   </si>
 </sst>
 </file>
@@ -833,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G137"/>
+  <dimension ref="A1:G143"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -3519,6 +3540,144 @@
         <v>115</v>
       </c>
       <c r="G137" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A138" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B138" t="s">
+        <v>139</v>
+      </c>
+      <c r="C138" t="s">
+        <v>113</v>
+      </c>
+      <c r="D138" s="2">
+        <v>12756800</v>
+      </c>
+      <c r="E138" t="s">
+        <v>114</v>
+      </c>
+      <c r="F138" t="s">
+        <v>115</v>
+      </c>
+      <c r="G138" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A139" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B139" t="s">
+        <v>140</v>
+      </c>
+      <c r="C139" t="s">
+        <v>113</v>
+      </c>
+      <c r="D139" s="2">
+        <v>2087500</v>
+      </c>
+      <c r="E139" t="s">
+        <v>125</v>
+      </c>
+      <c r="F139" s="2">
+        <v>2080000</v>
+      </c>
+      <c r="G139" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A140" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B140" t="s">
+        <v>141</v>
+      </c>
+      <c r="C140" t="s">
+        <v>113</v>
+      </c>
+      <c r="D140" s="2">
+        <v>13600300</v>
+      </c>
+      <c r="E140" t="s">
+        <v>142</v>
+      </c>
+      <c r="F140" s="2">
+        <v>12934000</v>
+      </c>
+      <c r="G140" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A141" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B141" t="s">
+        <v>143</v>
+      </c>
+      <c r="C141" t="s">
+        <v>113</v>
+      </c>
+      <c r="D141" s="2">
+        <v>160000</v>
+      </c>
+      <c r="E141" t="s">
+        <v>130</v>
+      </c>
+      <c r="F141" t="s">
+        <v>115</v>
+      </c>
+      <c r="G141" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A142" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B142" t="s">
+        <v>144</v>
+      </c>
+      <c r="C142" t="s">
+        <v>125</v>
+      </c>
+      <c r="D142" s="2">
+        <v>1440000</v>
+      </c>
+      <c r="E142" t="s">
+        <v>113</v>
+      </c>
+      <c r="F142" t="s">
+        <v>115</v>
+      </c>
+      <c r="G142" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A143" s="1">
+        <v>45818</v>
+      </c>
+      <c r="B143" t="s">
+        <v>145</v>
+      </c>
+      <c r="C143" t="s">
+        <v>142</v>
+      </c>
+      <c r="D143" s="2">
+        <v>1840800</v>
+      </c>
+      <c r="E143" t="s">
+        <v>113</v>
+      </c>
+      <c r="F143" t="s">
+        <v>115</v>
+      </c>
+      <c r="G143" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 11.06.2025 07:36
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39920400-FD7E-4F36-B782-1EA50BD09E83}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B4C29C8-0E65-40D5-9DA4-418395419671}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="154">
   <si>
     <t>Datum</t>
   </si>
@@ -477,19 +477,49 @@
   </si>
   <si>
     <t xml:space="preserve"> K. Müller</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Neuhaus</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maza</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Trimmel</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Gomis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Vasilj</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Hennrich</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Can</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Stergiou</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -512,10 +542,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -854,7 +887,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G143"/>
+  <dimension ref="A1:G156"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -3596,19 +3629,19 @@
       <c r="B140" t="s">
         <v>141</v>
       </c>
-      <c r="C140" t="s">
+      <c r="C140" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D140" s="2">
+      <c r="D140">
         <v>13600300</v>
       </c>
-      <c r="E140" t="s">
+      <c r="E140" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="F140" s="2">
+      <c r="F140">
         <v>12934000</v>
       </c>
-      <c r="G140" t="s">
+      <c r="G140" s="1" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3619,19 +3652,19 @@
       <c r="B141" t="s">
         <v>143</v>
       </c>
-      <c r="C141" t="s">
+      <c r="C141" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="D141" s="2">
+      <c r="D141">
         <v>160000</v>
       </c>
-      <c r="E141" t="s">
+      <c r="E141" s="1" t="s">
         <v>130</v>
       </c>
       <c r="F141" t="s">
         <v>115</v>
       </c>
-      <c r="G141" t="s">
+      <c r="G141" s="1" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3642,19 +3675,19 @@
       <c r="B142" t="s">
         <v>144</v>
       </c>
-      <c r="C142" t="s">
+      <c r="C142" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D142" s="2">
+      <c r="D142">
         <v>1440000</v>
       </c>
-      <c r="E142" t="s">
+      <c r="E142" s="1" t="s">
         <v>113</v>
       </c>
       <c r="F142" t="s">
         <v>115</v>
       </c>
-      <c r="G142" t="s">
+      <c r="G142" s="1" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3665,21 +3698,220 @@
       <c r="B143" t="s">
         <v>145</v>
       </c>
-      <c r="C143" t="s">
+      <c r="C143" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="D143" s="2">
+      <c r="D143">
         <v>1840800</v>
       </c>
-      <c r="E143" t="s">
+      <c r="E143" s="1" t="s">
         <v>113</v>
       </c>
       <c r="F143" t="s">
         <v>115</v>
       </c>
-      <c r="G143" t="s">
-        <v>115</v>
-      </c>
+      <c r="G143" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A144" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B144" t="s">
+        <v>146</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D144">
+        <v>3167000</v>
+      </c>
+      <c r="E144" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F144">
+        <v>2861100</v>
+      </c>
+      <c r="G144" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A145" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B145" t="s">
+        <v>147</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D145">
+        <v>9575555</v>
+      </c>
+      <c r="E145" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="F145">
+        <v>9564000</v>
+      </c>
+      <c r="G145" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A146" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B146" t="s">
+        <v>148</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D146">
+        <v>2121323</v>
+      </c>
+      <c r="E146" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="F146" t="s">
+        <v>115</v>
+      </c>
+      <c r="G146" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A147" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B147" t="s">
+        <v>149</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="D147">
+        <v>1477000</v>
+      </c>
+      <c r="E147" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="F147" t="s">
+        <v>115</v>
+      </c>
+      <c r="G147" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A148" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B148" t="s">
+        <v>150</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D148">
+        <v>3161300</v>
+      </c>
+      <c r="E148" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F148" t="s">
+        <v>115</v>
+      </c>
+      <c r="G148" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A149" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B149" t="s">
+        <v>151</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D149">
+        <v>168000</v>
+      </c>
+      <c r="E149" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F149" t="s">
+        <v>115</v>
+      </c>
+      <c r="G149" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A150" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B150" t="s">
+        <v>152</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D150">
+        <v>3520000</v>
+      </c>
+      <c r="E150" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F150" t="s">
+        <v>115</v>
+      </c>
+      <c r="G150" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A151" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B151" t="s">
+        <v>153</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="D151">
+        <v>1500000</v>
+      </c>
+      <c r="E151" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="F151" t="s">
+        <v>115</v>
+      </c>
+      <c r="G151" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A152" s="3"/>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A153" s="3"/>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A154" s="3"/>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A155" s="3"/>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A156" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 12.06.2025 07:45
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A13FDB97-07F6-47C2-BDE8-E8D789A8FD5C}"/>
+  <xr:revisionPtr revIDLastSave="56" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6843F368-8724-47D5-8797-ADAD5BE367FE}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="156">
   <si>
     <t>Datum</t>
   </si>
@@ -501,6 +501,12 @@
   </si>
   <si>
     <t xml:space="preserve"> Stergiou</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Skarke</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Elfadli</t>
   </si>
 </sst>
 </file>
@@ -874,7 +880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G151"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -3708,19 +3714,19 @@
       <c r="B144" t="s">
         <v>146</v>
       </c>
-      <c r="C144" s="1" t="s">
+      <c r="C144" t="s">
         <v>113</v>
       </c>
-      <c r="D144">
+      <c r="D144" s="2">
         <v>3167000</v>
       </c>
-      <c r="E144" s="1" t="s">
+      <c r="E144" t="s">
         <v>130</v>
       </c>
-      <c r="F144">
+      <c r="F144" s="2">
         <v>2861100</v>
       </c>
-      <c r="G144" s="1" t="s">
+      <c r="G144" t="s">
         <v>125</v>
       </c>
     </row>
@@ -3731,19 +3737,19 @@
       <c r="B145" t="s">
         <v>147</v>
       </c>
-      <c r="C145" s="1" t="s">
+      <c r="C145" t="s">
         <v>113</v>
       </c>
-      <c r="D145">
+      <c r="D145" s="2">
         <v>9575555</v>
       </c>
-      <c r="E145" s="1" t="s">
+      <c r="E145" t="s">
         <v>125</v>
       </c>
-      <c r="F145">
+      <c r="F145" s="2">
         <v>9564000</v>
       </c>
-      <c r="G145" s="1" t="s">
+      <c r="G145" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3754,19 +3760,19 @@
       <c r="B146" t="s">
         <v>148</v>
       </c>
-      <c r="C146" s="1" t="s">
+      <c r="C146" t="s">
         <v>113</v>
       </c>
-      <c r="D146">
+      <c r="D146" s="2">
         <v>2121323</v>
       </c>
-      <c r="E146" s="1" t="s">
+      <c r="E146" t="s">
         <v>121</v>
       </c>
       <c r="F146" t="s">
         <v>115</v>
       </c>
-      <c r="G146" s="1" t="s">
+      <c r="G146" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3777,19 +3783,19 @@
       <c r="B147" t="s">
         <v>149</v>
       </c>
-      <c r="C147" s="1" t="s">
+      <c r="C147" t="s">
         <v>113</v>
       </c>
-      <c r="D147">
+      <c r="D147" s="2">
         <v>1477000</v>
       </c>
-      <c r="E147" s="1" t="s">
+      <c r="E147" t="s">
         <v>130</v>
       </c>
       <c r="F147" t="s">
         <v>115</v>
       </c>
-      <c r="G147" s="1" t="s">
+      <c r="G147" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3800,19 +3806,19 @@
       <c r="B148" t="s">
         <v>150</v>
       </c>
-      <c r="C148" s="1" t="s">
+      <c r="C148" t="s">
         <v>114</v>
       </c>
-      <c r="D148">
+      <c r="D148" s="2">
         <v>3161300</v>
       </c>
-      <c r="E148" s="1" t="s">
+      <c r="E148" t="s">
         <v>113</v>
       </c>
       <c r="F148" t="s">
         <v>115</v>
       </c>
-      <c r="G148" s="1" t="s">
+      <c r="G148" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3823,19 +3829,19 @@
       <c r="B149" t="s">
         <v>151</v>
       </c>
-      <c r="C149" s="1" t="s">
+      <c r="C149" t="s">
         <v>114</v>
       </c>
-      <c r="D149">
+      <c r="D149" s="2">
         <v>168000</v>
       </c>
-      <c r="E149" s="1" t="s">
+      <c r="E149" t="s">
         <v>113</v>
       </c>
       <c r="F149" t="s">
         <v>115</v>
       </c>
-      <c r="G149" s="1" t="s">
+      <c r="G149" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3846,19 +3852,19 @@
       <c r="B150" t="s">
         <v>152</v>
       </c>
-      <c r="C150" s="1" t="s">
+      <c r="C150" t="s">
         <v>114</v>
       </c>
-      <c r="D150">
+      <c r="D150" s="2">
         <v>3520000</v>
       </c>
-      <c r="E150" s="1" t="s">
+      <c r="E150" t="s">
         <v>113</v>
       </c>
       <c r="F150" t="s">
         <v>115</v>
       </c>
-      <c r="G150" s="1" t="s">
+      <c r="G150" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3867,21 +3873,90 @@
         <v>45819</v>
       </c>
       <c r="B151" t="s">
+        <v>154</v>
+      </c>
+      <c r="C151" t="s">
+        <v>130</v>
+      </c>
+      <c r="D151" s="2">
+        <v>1407600</v>
+      </c>
+      <c r="E151" t="s">
+        <v>113</v>
+      </c>
+      <c r="F151" t="s">
+        <v>115</v>
+      </c>
+      <c r="G151" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A152" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B152" t="s">
         <v>153</v>
       </c>
-      <c r="C151" s="1" t="s">
+      <c r="C152" t="s">
         <v>114</v>
       </c>
-      <c r="D151">
+      <c r="D152" s="2">
         <v>1500000</v>
       </c>
-      <c r="E151" s="1" t="s">
+      <c r="E152" t="s">
         <v>132</v>
       </c>
-      <c r="F151" t="s">
-        <v>115</v>
-      </c>
-      <c r="G151" s="1" t="s">
+      <c r="F152" t="s">
+        <v>115</v>
+      </c>
+      <c r="G152" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A153" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B153" t="s">
+        <v>155</v>
+      </c>
+      <c r="C153" t="s">
+        <v>114</v>
+      </c>
+      <c r="D153" s="2">
+        <v>3800000</v>
+      </c>
+      <c r="E153" t="s">
+        <v>132</v>
+      </c>
+      <c r="F153" t="s">
+        <v>115</v>
+      </c>
+      <c r="G153" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A154" s="1">
+        <v>45819</v>
+      </c>
+      <c r="B154" t="s">
+        <v>134</v>
+      </c>
+      <c r="C154" t="s">
+        <v>117</v>
+      </c>
+      <c r="D154" s="2">
+        <v>4900000</v>
+      </c>
+      <c r="E154" t="s">
+        <v>132</v>
+      </c>
+      <c r="F154" t="s">
+        <v>115</v>
+      </c>
+      <c r="G154" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 12.06.2025 07:47
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6843F368-8724-47D5-8797-ADAD5BE367FE}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FBC244B-78A5-4B6F-8B36-AB75342B7345}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="159">
   <si>
     <t>Datum</t>
   </si>
@@ -507,6 +507,15 @@
   </si>
   <si>
     <t xml:space="preserve"> Elfadli</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Millot</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Noll</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Süle</t>
   </si>
 </sst>
 </file>
@@ -561,6 +570,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -880,7 +893,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G158"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -3957,6 +3970,98 @@
         <v>115</v>
       </c>
       <c r="G154" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A155" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B155" t="s">
+        <v>156</v>
+      </c>
+      <c r="C155" t="s">
+        <v>113</v>
+      </c>
+      <c r="D155" s="2">
+        <v>6750000</v>
+      </c>
+      <c r="E155" t="s">
+        <v>120</v>
+      </c>
+      <c r="F155" s="2">
+        <v>6700000</v>
+      </c>
+      <c r="G155" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A156" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B156" t="s">
+        <v>157</v>
+      </c>
+      <c r="C156" t="s">
+        <v>113</v>
+      </c>
+      <c r="D156" s="2">
+        <v>164000</v>
+      </c>
+      <c r="E156" t="s">
+        <v>114</v>
+      </c>
+      <c r="F156" s="2">
+        <v>161000</v>
+      </c>
+      <c r="G156" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A157" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B157" t="s">
+        <v>158</v>
+      </c>
+      <c r="C157" t="s">
+        <v>113</v>
+      </c>
+      <c r="D157" s="2">
+        <v>4710001</v>
+      </c>
+      <c r="E157" t="s">
+        <v>117</v>
+      </c>
+      <c r="F157" s="2">
+        <v>4679509</v>
+      </c>
+      <c r="G157" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A158" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B158" t="s">
+        <v>122</v>
+      </c>
+      <c r="C158" t="s">
+        <v>117</v>
+      </c>
+      <c r="D158" s="2">
+        <v>280000</v>
+      </c>
+      <c r="E158" t="s">
+        <v>113</v>
+      </c>
+      <c r="F158" t="s">
+        <v>115</v>
+      </c>
+      <c r="G158" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 12.06.2025 07:50
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FBC244B-78A5-4B6F-8B36-AB75342B7345}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F884CE8-7E88-44AF-AC10-D71DC7F57017}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -3975,7 +3975,7 @@
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A155" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B155" t="s">
         <v>156</v>
@@ -3998,7 +3998,7 @@
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A156" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B156" t="s">
         <v>157</v>
@@ -4021,7 +4021,7 @@
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A157" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B157" t="s">
         <v>158</v>
@@ -4044,7 +4044,7 @@
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A158" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B158" t="s">
         <v>122</v>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 12.06.2025 10:41
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F884CE8-7E88-44AF-AC10-D71DC7F57017}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A65D2398-45FD-406C-9F92-5855B240ADEA}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="164">
   <si>
     <t>Datum</t>
   </si>
@@ -516,6 +516,21 @@
   </si>
   <si>
     <t xml:space="preserve"> Süle</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ouédraogo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Zetterer</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Traoré</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Beste</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sander</t>
   </si>
 </sst>
 </file>
@@ -893,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G158"/>
+  <dimension ref="A1:G164"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -4062,6 +4077,144 @@
         <v>115</v>
       </c>
       <c r="G158" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A159" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B159" t="s">
+        <v>140</v>
+      </c>
+      <c r="C159" t="s">
+        <v>125</v>
+      </c>
+      <c r="D159" s="2">
+        <v>2114600</v>
+      </c>
+      <c r="E159" t="s">
+        <v>113</v>
+      </c>
+      <c r="F159" t="s">
+        <v>115</v>
+      </c>
+      <c r="G159" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A160" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B160" t="s">
+        <v>159</v>
+      </c>
+      <c r="C160" t="s">
+        <v>125</v>
+      </c>
+      <c r="D160" s="2">
+        <v>2069600</v>
+      </c>
+      <c r="E160" t="s">
+        <v>113</v>
+      </c>
+      <c r="F160" t="s">
+        <v>115</v>
+      </c>
+      <c r="G160" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A161" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B161" t="s">
+        <v>160</v>
+      </c>
+      <c r="C161" t="s">
+        <v>142</v>
+      </c>
+      <c r="D161" s="2">
+        <v>2667000</v>
+      </c>
+      <c r="E161" t="s">
+        <v>113</v>
+      </c>
+      <c r="F161" t="s">
+        <v>115</v>
+      </c>
+      <c r="G161" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A162" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B162" t="s">
+        <v>161</v>
+      </c>
+      <c r="C162" t="s">
+        <v>142</v>
+      </c>
+      <c r="D162" s="2">
+        <v>1326000</v>
+      </c>
+      <c r="E162" t="s">
+        <v>113</v>
+      </c>
+      <c r="F162" t="s">
+        <v>115</v>
+      </c>
+      <c r="G162" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A163" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B163" t="s">
+        <v>162</v>
+      </c>
+      <c r="C163" t="s">
+        <v>114</v>
+      </c>
+      <c r="D163" s="2">
+        <v>3450000</v>
+      </c>
+      <c r="E163" t="s">
+        <v>113</v>
+      </c>
+      <c r="F163" t="s">
+        <v>115</v>
+      </c>
+      <c r="G163" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A164" s="1">
+        <v>43994</v>
+      </c>
+      <c r="B164" t="s">
+        <v>163</v>
+      </c>
+      <c r="C164" t="s">
+        <v>114</v>
+      </c>
+      <c r="D164" s="2">
+        <v>2270000</v>
+      </c>
+      <c r="E164" t="s">
+        <v>113</v>
+      </c>
+      <c r="F164" t="s">
+        <v>115</v>
+      </c>
+      <c r="G164" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 12.06.2025 10:45
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A65D2398-45FD-406C-9F92-5855B240ADEA}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45AF8FBE-F98F-456C-876D-6FB3D1458074}"/>
   <bookViews>
     <workbookView xWindow="2110" yWindow="2130" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -4082,7 +4082,7 @@
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A159" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B159" t="s">
         <v>140</v>
@@ -4105,7 +4105,7 @@
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A160" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B160" t="s">
         <v>159</v>
@@ -4128,7 +4128,7 @@
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A161" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B161" t="s">
         <v>160</v>
@@ -4151,7 +4151,7 @@
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A162" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B162" t="s">
         <v>161</v>
@@ -4174,7 +4174,7 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A163" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B163" t="s">
         <v>162</v>
@@ -4197,7 +4197,7 @@
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A164" s="1">
-        <v>43994</v>
+        <v>45820</v>
       </c>
       <c r="B164" t="s">
         <v>163</v>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 13.06.2025 21:29
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="72" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08FC8C7D-0A3E-4B4C-9BDB-8572C022833B}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA4FBF9F-9622-4B57-9C6C-F772A0194641}"/>
   <bookViews>
-    <workbookView xWindow="16710" yWindow="2670" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
+    <workbookView xWindow="6660" yWindow="2700" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="173">
   <si>
     <t>Datum</t>
   </si>
@@ -555,6 +555,9 @@
   </si>
   <si>
     <t xml:space="preserve"> Höfler</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Schlager</t>
   </si>
 </sst>
 </file>
@@ -932,7 +935,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G173"/>
+  <dimension ref="A1:G175"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -4446,6 +4449,52 @@
         <v>115</v>
       </c>
       <c r="G173" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A174" s="1">
+        <v>43995</v>
+      </c>
+      <c r="B174" t="s">
+        <v>157</v>
+      </c>
+      <c r="C174" t="s">
+        <v>114</v>
+      </c>
+      <c r="D174" s="2">
+        <v>170000</v>
+      </c>
+      <c r="E174" t="s">
+        <v>113</v>
+      </c>
+      <c r="F174" t="s">
+        <v>115</v>
+      </c>
+      <c r="G174" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A175" s="1">
+        <v>43995</v>
+      </c>
+      <c r="B175" t="s">
+        <v>172</v>
+      </c>
+      <c r="C175" t="s">
+        <v>114</v>
+      </c>
+      <c r="D175" s="2">
+        <v>3759500</v>
+      </c>
+      <c r="E175" t="s">
+        <v>113</v>
+      </c>
+      <c r="F175" t="s">
+        <v>115</v>
+      </c>
+      <c r="G175" t="s">
         <v>115</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisches Update TM + Transfers - 13.06.2025 22:20
</commit_message>
<xml_diff>
--- a/TRANSFERS_all.xlsx
+++ b/TRANSFERS_all.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aecf56309e6168f4/Documents/comunio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA4FBF9F-9622-4B57-9C6C-F772A0194641}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="8_{ACF7F08C-8920-42E4-BDCF-07A3995E2ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37ECCDB4-0A82-4DA5-B731-CC1DA0058577}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="2700" windowWidth="28800" windowHeight="15370" xr2:uid="{10CFCFEB-EC74-443C-894F-626CD3E3CFC9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="172">
   <si>
     <t>Datum</t>
   </si>
@@ -318,9 +318,6 @@
   </si>
   <si>
     <t>Pyrka</t>
-  </si>
-  <si>
-    <t>Hranáč (annulliert)</t>
   </si>
   <si>
     <t>Diehl</t>
@@ -935,7 +932,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA36D7CE-3FEC-4018-BA71-853D1DD34D87}">
-  <dimension ref="A1:G175"/>
+  <dimension ref="A1:G174"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="43" bestFit="1" customWidth="1"/>
@@ -952,10 +949,10 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" t="s">
         <v>110</v>
-      </c>
-      <c r="E1" t="s">
-        <v>111</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -969,7 +966,7 @@
         <v>45805</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
         <v>19</v>
@@ -986,7 +983,7 @@
         <v>45805</v>
       </c>
       <c r="B3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -1020,7 +1017,7 @@
         <v>45805</v>
       </c>
       <c r="B5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -1037,7 +1034,7 @@
         <v>45805</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -1054,7 +1051,7 @@
         <v>45806</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
         <v>6</v>
@@ -1094,7 +1091,7 @@
         <v>45806</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -1157,7 +1154,7 @@
         <v>45806</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
         <v>6</v>
@@ -1180,7 +1177,7 @@
         <v>45806</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
         <v>6</v>
@@ -1237,7 +1234,7 @@
         <v>45806</v>
       </c>
       <c r="B16" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C16" t="s">
         <v>6</v>
@@ -1283,7 +1280,7 @@
         <v>45806</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
         <v>6</v>
@@ -1300,7 +1297,7 @@
         <v>45806</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
@@ -1317,7 +1314,7 @@
         <v>45806</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
@@ -1334,7 +1331,7 @@
         <v>45806</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C21" t="s">
         <v>7</v>
@@ -1351,7 +1348,7 @@
         <v>45806</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
@@ -1368,7 +1365,7 @@
         <v>45806</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
@@ -1385,7 +1382,7 @@
         <v>45806</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C24" t="s">
         <v>24</v>
@@ -1402,7 +1399,7 @@
         <v>45807</v>
       </c>
       <c r="B25" t="s">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s">
         <v>6</v>
@@ -1412,6 +1409,12 @@
       </c>
       <c r="E25" t="s">
         <v>8</v>
+      </c>
+      <c r="F25" s="2">
+        <v>165000</v>
+      </c>
+      <c r="G25" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
@@ -1419,39 +1422,33 @@
         <v>45807</v>
       </c>
       <c r="B26" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="C26" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="2">
-        <v>1660000</v>
+        <v>250008</v>
       </c>
       <c r="E26" t="s">
-        <v>8</v>
-      </c>
-      <c r="F26" s="2">
-        <v>165000</v>
-      </c>
-      <c r="G26" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
-        <v>45807</v>
+        <v>45808</v>
       </c>
       <c r="B27" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="C27" t="s">
         <v>6</v>
       </c>
       <c r="D27" s="2">
-        <v>250008</v>
+        <v>15000000</v>
       </c>
       <c r="E27" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
@@ -1459,16 +1456,22 @@
         <v>45808</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
         <v>6</v>
       </c>
       <c r="D28" s="2">
-        <v>15000000</v>
+        <v>3105003</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>7</v>
+      </c>
+      <c r="F28" s="2">
+        <v>2947500</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
@@ -1476,22 +1479,16 @@
         <v>45808</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
         <v>6</v>
       </c>
       <c r="D29" s="2">
-        <v>3105003</v>
+        <v>180000</v>
       </c>
       <c r="E29" t="s">
-        <v>7</v>
-      </c>
-      <c r="F29" s="2">
-        <v>2947500</v>
-      </c>
-      <c r="G29" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
@@ -1499,16 +1496,22 @@
         <v>45808</v>
       </c>
       <c r="B30" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="C30" t="s">
         <v>6</v>
       </c>
       <c r="D30" s="2">
-        <v>180000</v>
+        <v>10558000</v>
       </c>
       <c r="E30" t="s">
         <v>22</v>
+      </c>
+      <c r="F30" s="2">
+        <v>10000002</v>
+      </c>
+      <c r="G30" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -1516,22 +1519,22 @@
         <v>45808</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C31" t="s">
         <v>6</v>
       </c>
       <c r="D31" s="2">
-        <v>10558000</v>
+        <v>1255000</v>
       </c>
       <c r="E31" t="s">
         <v>22</v>
       </c>
       <c r="F31" s="2">
-        <v>10000002</v>
+        <v>1162000</v>
       </c>
       <c r="G31" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
@@ -1539,22 +1542,16 @@
         <v>45808</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="C32" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="2">
-        <v>1255000</v>
+        <v>420050</v>
       </c>
       <c r="E32" t="s">
-        <v>22</v>
-      </c>
-      <c r="F32" s="2">
-        <v>1162000</v>
-      </c>
-      <c r="G32" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
@@ -1562,16 +1559,22 @@
         <v>45808</v>
       </c>
       <c r="B33" t="s">
-        <v>57</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
         <v>6</v>
       </c>
       <c r="D33" s="2">
-        <v>420050</v>
+        <v>1230011</v>
       </c>
       <c r="E33" t="s">
-        <v>14</v>
+        <v>8</v>
+      </c>
+      <c r="F33" s="2">
+        <v>1200000</v>
+      </c>
+      <c r="G33" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
@@ -1579,22 +1582,16 @@
         <v>45808</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="C34" t="s">
         <v>6</v>
       </c>
       <c r="D34" s="2">
-        <v>1230011</v>
+        <v>9231900</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
-      </c>
-      <c r="F34" s="2">
-        <v>1200000</v>
-      </c>
-      <c r="G34" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
@@ -1602,16 +1599,22 @@
         <v>45808</v>
       </c>
       <c r="B35" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
         <v>6</v>
       </c>
       <c r="D35" s="2">
-        <v>9231900</v>
+        <v>1423233</v>
       </c>
       <c r="E35" t="s">
-        <v>8</v>
+        <v>24</v>
+      </c>
+      <c r="F35" s="2">
+        <v>1390000</v>
+      </c>
+      <c r="G35" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
@@ -1619,22 +1622,16 @@
         <v>45808</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="C36" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D36" s="2">
-        <v>1423233</v>
+        <v>589000</v>
       </c>
       <c r="E36" t="s">
-        <v>24</v>
-      </c>
-      <c r="F36" s="2">
-        <v>1390000</v>
-      </c>
-      <c r="G36" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.35">
@@ -1642,13 +1639,13 @@
         <v>45808</v>
       </c>
       <c r="B37" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="C37" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="2">
-        <v>589000</v>
+        <v>1515000</v>
       </c>
       <c r="E37" t="s">
         <v>6</v>
@@ -1656,19 +1653,25 @@
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
-        <v>45808</v>
+        <v>45809</v>
       </c>
       <c r="B38" t="s">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D38" s="2">
-        <v>1515000</v>
+        <v>566000</v>
       </c>
       <c r="E38" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="F38" s="2">
+        <v>543000</v>
+      </c>
+      <c r="G38" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
@@ -1676,22 +1679,22 @@
         <v>45809</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="C39" t="s">
         <v>6</v>
       </c>
       <c r="D39" s="2">
-        <v>566000</v>
+        <v>4135353</v>
       </c>
       <c r="E39" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="F39" s="2">
-        <v>543000</v>
+        <v>3500000</v>
       </c>
       <c r="G39" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.35">
@@ -1699,22 +1702,16 @@
         <v>45809</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C40" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D40" s="2">
-        <v>4135353</v>
+        <v>12852000</v>
       </c>
       <c r="E40" t="s">
-        <v>24</v>
-      </c>
-      <c r="F40" s="2">
-        <v>3500000</v>
-      </c>
-      <c r="G40" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.35">
@@ -1722,13 +1719,13 @@
         <v>45809</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C41" t="s">
         <v>7</v>
       </c>
       <c r="D41" s="2">
-        <v>12852000</v>
+        <v>218400</v>
       </c>
       <c r="E41" t="s">
         <v>6</v>
@@ -1739,13 +1736,13 @@
         <v>45809</v>
       </c>
       <c r="B42" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" s="2">
-        <v>218400</v>
+        <v>197600</v>
       </c>
       <c r="E42" t="s">
         <v>6</v>
@@ -1756,13 +1753,13 @@
         <v>45809</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C43" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="D43" s="2">
-        <v>197600</v>
+        <v>188100</v>
       </c>
       <c r="E43" t="s">
         <v>6</v>
@@ -1773,13 +1770,13 @@
         <v>45809</v>
       </c>
       <c r="B44" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C44" t="s">
         <v>24</v>
       </c>
       <c r="D44" s="2">
-        <v>188100</v>
+        <v>426400</v>
       </c>
       <c r="E44" t="s">
         <v>6</v>
@@ -1790,13 +1787,13 @@
         <v>45809</v>
       </c>
       <c r="B45" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="C45" t="s">
         <v>24</v>
       </c>
       <c r="D45" s="2">
-        <v>426400</v>
+        <v>1312500</v>
       </c>
       <c r="E45" t="s">
         <v>6</v>
@@ -1807,13 +1804,13 @@
         <v>45809</v>
       </c>
       <c r="B46" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C46" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D46" s="2">
-        <v>1312500</v>
+        <v>6468800</v>
       </c>
       <c r="E46" t="s">
         <v>6</v>
@@ -1824,13 +1821,13 @@
         <v>45809</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" s="2">
-        <v>6468800</v>
+        <v>2793000</v>
       </c>
       <c r="E47" t="s">
         <v>6</v>
@@ -1841,13 +1838,13 @@
         <v>45809</v>
       </c>
       <c r="B48" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" s="2">
-        <v>2793000</v>
+        <v>1888700</v>
       </c>
       <c r="E48" t="s">
         <v>6</v>
@@ -1858,13 +1855,13 @@
         <v>45809</v>
       </c>
       <c r="B49" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D49" s="2">
-        <v>1888700</v>
+        <v>1639300</v>
       </c>
       <c r="E49" t="s">
         <v>6</v>
@@ -1875,13 +1872,13 @@
         <v>45809</v>
       </c>
       <c r="B50" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C50" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D50" s="2">
-        <v>1639300</v>
+        <v>217800</v>
       </c>
       <c r="E50" t="s">
         <v>6</v>
@@ -1892,13 +1889,13 @@
         <v>45809</v>
       </c>
       <c r="B51" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" s="2">
-        <v>217800</v>
+        <v>273000</v>
       </c>
       <c r="E51" t="s">
         <v>6</v>
@@ -1906,19 +1903,25 @@
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
-        <v>45809</v>
+        <v>45810</v>
       </c>
       <c r="B52" t="s">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="C52" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="D52" s="2">
-        <v>273000</v>
+        <v>7755200</v>
       </c>
       <c r="E52" t="s">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="F52" s="2">
+        <v>7300000</v>
+      </c>
+      <c r="G52" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.35">
@@ -1926,22 +1929,22 @@
         <v>45810</v>
       </c>
       <c r="B53" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C53" t="s">
         <v>6</v>
       </c>
       <c r="D53" s="2">
-        <v>7755200</v>
+        <v>4123233</v>
       </c>
       <c r="E53" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F53" s="2">
-        <v>7300000</v>
+        <v>3100000</v>
       </c>
       <c r="G53" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.35">
@@ -1949,22 +1952,16 @@
         <v>45810</v>
       </c>
       <c r="B54" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
         <v>6</v>
       </c>
       <c r="D54" s="2">
-        <v>4123233</v>
+        <v>160033</v>
       </c>
       <c r="E54" t="s">
-        <v>24</v>
-      </c>
-      <c r="F54" s="2">
-        <v>3100000</v>
-      </c>
-      <c r="G54" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.35">
@@ -1972,16 +1969,22 @@
         <v>45810</v>
       </c>
       <c r="B55" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="C55" t="s">
         <v>6</v>
       </c>
       <c r="D55" s="2">
-        <v>160033</v>
+        <v>2850005</v>
       </c>
       <c r="E55" t="s">
-        <v>22</v>
+        <v>7</v>
+      </c>
+      <c r="F55" s="2">
+        <v>2700000</v>
+      </c>
+      <c r="G55" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.35">
@@ -1989,22 +1992,22 @@
         <v>45810</v>
       </c>
       <c r="B56" t="s">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="C56" t="s">
         <v>6</v>
       </c>
       <c r="D56" s="2">
-        <v>2850005</v>
+        <v>456005</v>
       </c>
       <c r="E56" t="s">
         <v>7</v>
       </c>
       <c r="F56" s="2">
-        <v>2700000</v>
+        <v>393000</v>
       </c>
       <c r="G56" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.35">
@@ -2012,22 +2015,16 @@
         <v>45810</v>
       </c>
       <c r="B57" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="C57" t="s">
         <v>6</v>
       </c>
       <c r="D57" s="2">
-        <v>456005</v>
+        <v>230000</v>
       </c>
       <c r="E57" t="s">
-        <v>7</v>
-      </c>
-      <c r="F57" s="2">
-        <v>393000</v>
-      </c>
-      <c r="G57" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.35">
@@ -2035,16 +2032,22 @@
         <v>45810</v>
       </c>
       <c r="B58" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="C58" t="s">
         <v>6</v>
       </c>
       <c r="D58" s="2">
-        <v>230000</v>
+        <v>14211000</v>
       </c>
       <c r="E58" t="s">
-        <v>11</v>
+        <v>22</v>
+      </c>
+      <c r="F58" s="2">
+        <v>13640008</v>
+      </c>
+      <c r="G58" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.35">
@@ -2052,22 +2055,16 @@
         <v>45810</v>
       </c>
       <c r="B59" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C59" t="s">
         <v>6</v>
       </c>
       <c r="D59" s="2">
-        <v>14211000</v>
+        <v>262000</v>
       </c>
       <c r="E59" t="s">
         <v>22</v>
-      </c>
-      <c r="F59" s="2">
-        <v>13640008</v>
-      </c>
-      <c r="G59" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.35">
@@ -2075,16 +2072,16 @@
         <v>45810</v>
       </c>
       <c r="B60" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C60" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D60" s="2">
-        <v>262000</v>
+        <v>4268000</v>
       </c>
       <c r="E60" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.35">
@@ -2092,13 +2089,13 @@
         <v>45810</v>
       </c>
       <c r="B61" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C61" t="s">
         <v>24</v>
       </c>
       <c r="D61" s="2">
-        <v>4268000</v>
+        <v>163200</v>
       </c>
       <c r="E61" t="s">
         <v>6</v>
@@ -2109,13 +2106,13 @@
         <v>45810</v>
       </c>
       <c r="B62" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C62" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="D62" s="2">
-        <v>163200</v>
+        <v>210000</v>
       </c>
       <c r="E62" t="s">
         <v>6</v>
@@ -2126,13 +2123,13 @@
         <v>45810</v>
       </c>
       <c r="B63" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C63" t="s">
         <v>14</v>
       </c>
       <c r="D63" s="2">
-        <v>210000</v>
+        <v>285600</v>
       </c>
       <c r="E63" t="s">
         <v>6</v>
@@ -2143,13 +2140,13 @@
         <v>45810</v>
       </c>
       <c r="B64" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C64" t="s">
         <v>14</v>
       </c>
       <c r="D64" s="2">
-        <v>285600</v>
+        <v>183600</v>
       </c>
       <c r="E64" t="s">
         <v>6</v>
@@ -2160,13 +2157,13 @@
         <v>45810</v>
       </c>
       <c r="B65" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C65" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D65" s="2">
-        <v>183600</v>
+        <v>1060900</v>
       </c>
       <c r="E65" t="s">
         <v>6</v>
@@ -2177,13 +2174,13 @@
         <v>45810</v>
       </c>
       <c r="B66" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C66" t="s">
         <v>22</v>
       </c>
       <c r="D66" s="2">
-        <v>1060900</v>
+        <v>193800</v>
       </c>
       <c r="E66" t="s">
         <v>6</v>
@@ -2194,13 +2191,13 @@
         <v>45810</v>
       </c>
       <c r="B67" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C67" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D67" s="2">
-        <v>193800</v>
+        <v>9061500</v>
       </c>
       <c r="E67" t="s">
         <v>6</v>
@@ -2211,33 +2208,39 @@
         <v>45810</v>
       </c>
       <c r="B68" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C68" t="s">
         <v>8</v>
       </c>
       <c r="D68" s="2">
-        <v>9061500</v>
+        <v>1500000</v>
       </c>
       <c r="E68" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
-        <v>45810</v>
+        <v>45811</v>
       </c>
       <c r="B69" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="C69" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" s="2">
+        <v>1200000</v>
+      </c>
+      <c r="E69" t="s">
+        <v>34</v>
+      </c>
+      <c r="F69" s="2">
+        <v>1110000</v>
+      </c>
+      <c r="G69" t="s">
         <v>8</v>
-      </c>
-      <c r="D69" s="2">
-        <v>1500000</v>
-      </c>
-      <c r="E69" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.35">
@@ -2245,7 +2248,7 @@
         <v>45811</v>
       </c>
       <c r="B70" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C70" t="s">
         <v>6</v>
@@ -2257,7 +2260,7 @@
         <v>34</v>
       </c>
       <c r="F70" s="2">
-        <v>1110000</v>
+        <v>1185000</v>
       </c>
       <c r="G70" t="s">
         <v>8</v>
@@ -2268,22 +2271,16 @@
         <v>45811</v>
       </c>
       <c r="B71" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C71" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D71" s="2">
-        <v>1200000</v>
+        <v>388500</v>
       </c>
       <c r="E71" t="s">
-        <v>34</v>
-      </c>
-      <c r="F71" s="2">
-        <v>1185000</v>
-      </c>
-      <c r="G71" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.35">
@@ -2291,13 +2288,13 @@
         <v>45811</v>
       </c>
       <c r="B72" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C72" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D72" s="2">
-        <v>388500</v>
+        <v>1449600</v>
       </c>
       <c r="E72" t="s">
         <v>6</v>
@@ -2308,13 +2305,13 @@
         <v>45811</v>
       </c>
       <c r="B73" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C73" t="s">
         <v>19</v>
       </c>
       <c r="D73" s="2">
-        <v>1449600</v>
+        <v>1726400</v>
       </c>
       <c r="E73" t="s">
         <v>6</v>
@@ -2325,13 +2322,13 @@
         <v>45811</v>
       </c>
       <c r="B74" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C74" t="s">
         <v>19</v>
       </c>
       <c r="D74" s="2">
-        <v>1726400</v>
+        <v>1036800</v>
       </c>
       <c r="E74" t="s">
         <v>6</v>
@@ -2342,16 +2339,16 @@
         <v>45811</v>
       </c>
       <c r="B75" t="s">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C75" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D75" s="2">
-        <v>1036800</v>
+        <v>580000</v>
       </c>
       <c r="E75" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.35">
@@ -2359,13 +2356,13 @@
         <v>45811</v>
       </c>
       <c r="B76" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="C76" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D76" s="2">
-        <v>580000</v>
+        <v>180000</v>
       </c>
       <c r="E76" t="s">
         <v>7</v>
@@ -2373,19 +2370,19 @@
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
-        <v>45811</v>
+        <v>45812</v>
       </c>
       <c r="B77" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="C77" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="D77" s="2">
-        <v>180000</v>
+        <v>160000</v>
       </c>
       <c r="E77" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.35">
@@ -2393,16 +2390,22 @@
         <v>45812</v>
       </c>
       <c r="B78" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C78" t="s">
         <v>6</v>
       </c>
       <c r="D78" s="2">
-        <v>160000</v>
+        <v>670000</v>
       </c>
       <c r="E78" t="s">
-        <v>22</v>
+        <v>34</v>
+      </c>
+      <c r="F78" s="2">
+        <v>641089</v>
+      </c>
+      <c r="G78" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.35">
@@ -2410,22 +2413,22 @@
         <v>45812</v>
       </c>
       <c r="B79" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C79" t="s">
         <v>6</v>
       </c>
       <c r="D79" s="2">
-        <v>670000</v>
+        <v>3110005</v>
       </c>
       <c r="E79" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="F79" s="2">
-        <v>641089</v>
+        <v>2945500</v>
       </c>
       <c r="G79" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.35">
@@ -2433,19 +2436,19 @@
         <v>45812</v>
       </c>
       <c r="B80" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C80" t="s">
         <v>6</v>
       </c>
       <c r="D80" s="2">
-        <v>3110005</v>
+        <v>5350000</v>
       </c>
       <c r="E80" t="s">
         <v>7</v>
       </c>
       <c r="F80" s="2">
-        <v>2945500</v>
+        <v>4655700</v>
       </c>
       <c r="G80" t="s">
         <v>14</v>
@@ -2456,19 +2459,19 @@
         <v>45812</v>
       </c>
       <c r="B81" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C81" t="s">
         <v>6</v>
       </c>
       <c r="D81" s="2">
-        <v>5350000</v>
+        <v>6757575</v>
       </c>
       <c r="E81" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="F81" s="2">
-        <v>4655700</v>
+        <v>5545555</v>
       </c>
       <c r="G81" t="s">
         <v>14</v>
@@ -2479,22 +2482,22 @@
         <v>45812</v>
       </c>
       <c r="B82" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C82" t="s">
         <v>6</v>
       </c>
       <c r="D82" s="2">
-        <v>6757575</v>
+        <v>4123233</v>
       </c>
       <c r="E82" t="s">
         <v>24</v>
       </c>
       <c r="F82" s="2">
-        <v>5545555</v>
+        <v>4000000</v>
       </c>
       <c r="G82" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.35">
@@ -2502,19 +2505,19 @@
         <v>45812</v>
       </c>
       <c r="B83" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C83" t="s">
         <v>6</v>
       </c>
       <c r="D83" s="2">
-        <v>4123233</v>
+        <v>2150008</v>
       </c>
       <c r="E83" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="F83" s="2">
-        <v>4000000</v>
+        <v>1500000</v>
       </c>
       <c r="G83" t="s">
         <v>11</v>
@@ -2525,22 +2528,16 @@
         <v>45812</v>
       </c>
       <c r="B84" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C84" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D84" s="2">
-        <v>2150008</v>
+        <v>3097500</v>
       </c>
       <c r="E84" t="s">
-        <v>7</v>
-      </c>
-      <c r="F84" s="2">
-        <v>1500000</v>
-      </c>
-      <c r="G84" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.35">
@@ -2548,13 +2545,13 @@
         <v>45812</v>
       </c>
       <c r="B85" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C85" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D85" s="2">
-        <v>3097500</v>
+        <v>7266000</v>
       </c>
       <c r="E85" t="s">
         <v>6</v>
@@ -2565,13 +2562,13 @@
         <v>45812</v>
       </c>
       <c r="B86" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C86" t="s">
         <v>22</v>
       </c>
       <c r="D86" s="2">
-        <v>7266000</v>
+        <v>163200</v>
       </c>
       <c r="E86" t="s">
         <v>6</v>
@@ -2582,13 +2579,13 @@
         <v>45812</v>
       </c>
       <c r="B87" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C87" t="s">
         <v>22</v>
       </c>
       <c r="D87" s="2">
-        <v>163200</v>
+        <v>520000</v>
       </c>
       <c r="E87" t="s">
         <v>6</v>
@@ -2599,33 +2596,39 @@
         <v>45812</v>
       </c>
       <c r="B88" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C88" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D88" s="2">
-        <v>520000</v>
+        <v>5500000</v>
       </c>
       <c r="E88" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
-        <v>45812</v>
+        <v>45813</v>
       </c>
       <c r="B89" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="C89" t="s">
+        <v>6</v>
+      </c>
+      <c r="D89" s="2">
+        <v>4500000</v>
+      </c>
+      <c r="E89" t="s">
         <v>8</v>
       </c>
-      <c r="D89" s="2">
-        <v>5500000</v>
-      </c>
-      <c r="E89" t="s">
-        <v>19</v>
+      <c r="F89" s="2">
+        <v>4050008</v>
+      </c>
+      <c r="G89" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.35">
@@ -2633,22 +2636,22 @@
         <v>45813</v>
       </c>
       <c r="B90" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C90" t="s">
         <v>6</v>
       </c>
       <c r="D90" s="2">
-        <v>4500000</v>
+        <v>7390000</v>
       </c>
       <c r="E90" t="s">
+        <v>34</v>
+      </c>
+      <c r="F90" s="2">
+        <v>7150009</v>
+      </c>
+      <c r="G90" t="s">
         <v>8</v>
-      </c>
-      <c r="F90" s="2">
-        <v>4050008</v>
-      </c>
-      <c r="G90" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.35">
@@ -2656,22 +2659,16 @@
         <v>45813</v>
       </c>
       <c r="B91" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C91" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D91" s="2">
-        <v>7390000</v>
+        <v>1620000</v>
       </c>
       <c r="E91" t="s">
-        <v>34</v>
-      </c>
-      <c r="F91" s="2">
-        <v>7150009</v>
-      </c>
-      <c r="G91" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.35">
@@ -2679,13 +2676,13 @@
         <v>45813</v>
       </c>
       <c r="B92" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C92" t="s">
         <v>24</v>
       </c>
       <c r="D92" s="2">
-        <v>1620000</v>
+        <v>2028000</v>
       </c>
       <c r="E92" t="s">
         <v>6</v>
@@ -2696,13 +2693,13 @@
         <v>45813</v>
       </c>
       <c r="B93" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C93" t="s">
         <v>24</v>
       </c>
       <c r="D93" s="2">
-        <v>2028000</v>
+        <v>595200</v>
       </c>
       <c r="E93" t="s">
         <v>6</v>
@@ -2713,13 +2710,13 @@
         <v>45813</v>
       </c>
       <c r="B94" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C94" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D94" s="2">
-        <v>595200</v>
+        <v>470000</v>
       </c>
       <c r="E94" t="s">
         <v>6</v>
@@ -2730,13 +2727,13 @@
         <v>45813</v>
       </c>
       <c r="B95" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C95" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D95" s="2">
-        <v>470000</v>
+        <v>203700</v>
       </c>
       <c r="E95" t="s">
         <v>6</v>
@@ -2747,13 +2744,13 @@
         <v>45813</v>
       </c>
       <c r="B96" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C96" t="s">
         <v>11</v>
       </c>
       <c r="D96" s="2">
-        <v>203700</v>
+        <v>13020800</v>
       </c>
       <c r="E96" t="s">
         <v>6</v>
@@ -2764,13 +2761,13 @@
         <v>45813</v>
       </c>
       <c r="B97" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C97" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D97" s="2">
-        <v>13020800</v>
+        <v>199500</v>
       </c>
       <c r="E97" t="s">
         <v>6</v>
@@ -2781,13 +2778,13 @@
         <v>45813</v>
       </c>
       <c r="B98" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C98" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D98" s="2">
-        <v>199500</v>
+        <v>192000</v>
       </c>
       <c r="E98" t="s">
         <v>6</v>
@@ -2795,19 +2792,25 @@
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
-        <v>45813</v>
+        <v>45814</v>
       </c>
       <c r="B99" t="s">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="C99" t="s">
+        <v>6</v>
+      </c>
+      <c r="D99" s="2">
+        <v>3200000</v>
+      </c>
+      <c r="E99" t="s">
         <v>11</v>
       </c>
-      <c r="D99" s="2">
-        <v>192000</v>
-      </c>
-      <c r="E99" t="s">
-        <v>6</v>
+      <c r="F99" s="2">
+        <v>2600000</v>
+      </c>
+      <c r="G99" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.35">
@@ -2815,22 +2818,22 @@
         <v>45814</v>
       </c>
       <c r="B100" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C100" t="s">
         <v>6</v>
       </c>
       <c r="D100" s="2">
-        <v>3200000</v>
+        <v>1395200</v>
       </c>
       <c r="E100" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F100" s="2">
-        <v>2600000</v>
+        <v>1350005</v>
       </c>
       <c r="G100" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.35">
@@ -2838,19 +2841,19 @@
         <v>45814</v>
       </c>
       <c r="B101" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C101" t="s">
         <v>6</v>
       </c>
       <c r="D101" s="2">
-        <v>1395200</v>
+        <v>2555000</v>
       </c>
       <c r="E101" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F101" s="2">
-        <v>1350005</v>
+        <v>2550002</v>
       </c>
       <c r="G101" t="s">
         <v>7</v>
@@ -2861,22 +2864,22 @@
         <v>45814</v>
       </c>
       <c r="B102" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C102" t="s">
         <v>6</v>
       </c>
       <c r="D102" s="2">
-        <v>2555000</v>
+        <v>4536666</v>
       </c>
       <c r="E102" t="s">
+        <v>24</v>
+      </c>
+      <c r="F102" s="2">
+        <v>3777000</v>
+      </c>
+      <c r="G102" t="s">
         <v>22</v>
-      </c>
-      <c r="F102" s="2">
-        <v>2550002</v>
-      </c>
-      <c r="G102" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.35">
@@ -2884,22 +2887,22 @@
         <v>45814</v>
       </c>
       <c r="B103" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C103" t="s">
         <v>6</v>
       </c>
       <c r="D103" s="2">
-        <v>4536666</v>
+        <v>5355355</v>
       </c>
       <c r="E103" t="s">
         <v>24</v>
       </c>
       <c r="F103" s="2">
-        <v>3777000</v>
+        <v>4700000</v>
       </c>
       <c r="G103" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.35">
@@ -2907,21 +2910,15 @@
         <v>45814</v>
       </c>
       <c r="B104" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C104" t="s">
         <v>6</v>
       </c>
       <c r="D104" s="2">
-        <v>5355355</v>
+        <v>605009</v>
       </c>
       <c r="E104" t="s">
-        <v>24</v>
-      </c>
-      <c r="F104" s="2">
-        <v>4700000</v>
-      </c>
-      <c r="G104" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2930,16 +2927,22 @@
         <v>45814</v>
       </c>
       <c r="B105" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C105" t="s">
         <v>6</v>
       </c>
       <c r="D105" s="2">
-        <v>605009</v>
+        <v>800289</v>
       </c>
       <c r="E105" t="s">
         <v>8</v>
+      </c>
+      <c r="F105" s="2">
+        <v>800008</v>
+      </c>
+      <c r="G105" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.35">
@@ -2947,22 +2950,22 @@
         <v>45814</v>
       </c>
       <c r="B106" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C106" t="s">
         <v>6</v>
       </c>
       <c r="D106" s="2">
-        <v>800289</v>
+        <v>1685000</v>
       </c>
       <c r="E106" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F106" s="2">
-        <v>800008</v>
+        <v>1665123</v>
       </c>
       <c r="G106" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.35">
@@ -2970,22 +2973,16 @@
         <v>45814</v>
       </c>
       <c r="B107" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C107" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D107" s="2">
-        <v>1685000</v>
+        <v>164800</v>
       </c>
       <c r="E107" t="s">
-        <v>7</v>
-      </c>
-      <c r="F107" s="2">
-        <v>1665123</v>
-      </c>
-      <c r="G107" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.35">
@@ -2993,13 +2990,13 @@
         <v>45814</v>
       </c>
       <c r="B108" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C108" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D108" s="2">
-        <v>164800</v>
+        <v>450000</v>
       </c>
       <c r="E108" t="s">
         <v>6</v>
@@ -3010,13 +3007,13 @@
         <v>45814</v>
       </c>
       <c r="B109" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C109" t="s">
         <v>7</v>
       </c>
       <c r="D109" s="2">
-        <v>450000</v>
+        <v>462000</v>
       </c>
       <c r="E109" t="s">
         <v>6</v>
@@ -3024,19 +3021,25 @@
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
-        <v>45814</v>
+        <v>45815</v>
       </c>
       <c r="B110" t="s">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="C110" t="s">
+        <v>6</v>
+      </c>
+      <c r="D110" s="2">
+        <v>3110009</v>
+      </c>
+      <c r="E110" t="s">
         <v>7</v>
       </c>
-      <c r="D110" s="2">
-        <v>462000</v>
-      </c>
-      <c r="E110" t="s">
-        <v>6</v>
+      <c r="F110" s="2">
+        <v>3000000</v>
+      </c>
+      <c r="G110" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.35">
@@ -3044,19 +3047,19 @@
         <v>45815</v>
       </c>
       <c r="B111" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C111" t="s">
         <v>6</v>
       </c>
       <c r="D111" s="2">
-        <v>3110009</v>
+        <v>195008</v>
       </c>
       <c r="E111" t="s">
         <v>7</v>
       </c>
       <c r="F111" s="2">
-        <v>3000000</v>
+        <v>173000</v>
       </c>
       <c r="G111" t="s">
         <v>8</v>
@@ -3067,19 +3070,19 @@
         <v>45815</v>
       </c>
       <c r="B112" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C112" t="s">
         <v>6</v>
       </c>
       <c r="D112" s="2">
-        <v>195008</v>
+        <v>2221000</v>
       </c>
       <c r="E112" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F112" s="2">
-        <v>173000</v>
+        <v>2000000</v>
       </c>
       <c r="G112" t="s">
         <v>8</v>
@@ -3090,22 +3093,16 @@
         <v>45815</v>
       </c>
       <c r="B113" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C113" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D113" s="2">
-        <v>2221000</v>
+        <v>1713600</v>
       </c>
       <c r="E113" t="s">
-        <v>11</v>
-      </c>
-      <c r="F113" s="2">
-        <v>2000000</v>
-      </c>
-      <c r="G113" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.35">
@@ -3113,13 +3110,13 @@
         <v>45815</v>
       </c>
       <c r="B114" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C114" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D114" s="2">
-        <v>1713600</v>
+        <v>198000</v>
       </c>
       <c r="E114" t="s">
         <v>6</v>
@@ -3130,13 +3127,13 @@
         <v>45815</v>
       </c>
       <c r="B115" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C115" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D115" s="2">
-        <v>198000</v>
+        <v>5018400</v>
       </c>
       <c r="E115" t="s">
         <v>6</v>
@@ -3147,13 +3144,13 @@
         <v>45815</v>
       </c>
       <c r="B116" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C116" t="s">
         <v>7</v>
       </c>
       <c r="D116" s="2">
-        <v>5018400</v>
+        <v>1040000</v>
       </c>
       <c r="E116" t="s">
         <v>6</v>
@@ -3164,13 +3161,13 @@
         <v>45815</v>
       </c>
       <c r="B117" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C117" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D117" s="2">
-        <v>1040000</v>
+        <v>1060500</v>
       </c>
       <c r="E117" t="s">
         <v>6</v>
@@ -3178,19 +3175,25 @@
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
-        <v>45815</v>
+        <v>45816</v>
       </c>
       <c r="B118" t="s">
-        <v>17</v>
+        <v>111</v>
       </c>
       <c r="C118" t="s">
-        <v>14</v>
+        <v>112</v>
       </c>
       <c r="D118" s="2">
-        <v>1060500</v>
+        <v>6391777</v>
       </c>
       <c r="E118" t="s">
-        <v>6</v>
+        <v>113</v>
+      </c>
+      <c r="F118" t="s">
+        <v>114</v>
+      </c>
+      <c r="G118" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.35">
@@ -3198,22 +3201,22 @@
         <v>45816</v>
       </c>
       <c r="B119" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C119" t="s">
+        <v>112</v>
+      </c>
+      <c r="D119" s="2">
+        <v>3450001</v>
+      </c>
+      <c r="E119" t="s">
         <v>113</v>
       </c>
-      <c r="D119" s="2">
-        <v>6391777</v>
-      </c>
-      <c r="E119" t="s">
-        <v>114</v>
-      </c>
-      <c r="F119" t="s">
-        <v>115</v>
+      <c r="F119" s="2">
+        <v>3435011</v>
       </c>
       <c r="G119" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.35">
@@ -3221,22 +3224,22 @@
         <v>45816</v>
       </c>
       <c r="B120" t="s">
+        <v>117</v>
+      </c>
+      <c r="C120" t="s">
+        <v>112</v>
+      </c>
+      <c r="D120" s="2">
+        <v>1011001</v>
+      </c>
+      <c r="E120" t="s">
+        <v>113</v>
+      </c>
+      <c r="F120" s="2">
+        <v>965000</v>
+      </c>
+      <c r="G120" t="s">
         <v>116</v>
-      </c>
-      <c r="C120" t="s">
-        <v>113</v>
-      </c>
-      <c r="D120" s="2">
-        <v>3450001</v>
-      </c>
-      <c r="E120" t="s">
-        <v>114</v>
-      </c>
-      <c r="F120" s="2">
-        <v>3435011</v>
-      </c>
-      <c r="G120" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.35">
@@ -3247,19 +3250,19 @@
         <v>118</v>
       </c>
       <c r="C121" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D121" s="2">
-        <v>1011001</v>
+        <v>350000</v>
       </c>
       <c r="E121" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F121" s="2">
-        <v>965000</v>
+        <v>323233</v>
       </c>
       <c r="G121" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.35">
@@ -3267,22 +3270,22 @@
         <v>45816</v>
       </c>
       <c r="B122" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C122" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D122" s="2">
-        <v>350000</v>
+        <v>310000</v>
       </c>
       <c r="E122" t="s">
-        <v>120</v>
-      </c>
-      <c r="F122" s="2">
-        <v>323233</v>
+        <v>116</v>
+      </c>
+      <c r="F122" t="s">
+        <v>114</v>
       </c>
       <c r="G122" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.35">
@@ -3293,19 +3296,19 @@
         <v>122</v>
       </c>
       <c r="C123" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D123" s="2">
-        <v>310000</v>
+        <v>5000000</v>
       </c>
       <c r="E123" t="s">
-        <v>117</v>
-      </c>
-      <c r="F123" t="s">
-        <v>115</v>
+        <v>116</v>
+      </c>
+      <c r="F123" s="2">
+        <v>4112122</v>
       </c>
       <c r="G123" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.35">
@@ -3316,19 +3319,19 @@
         <v>123</v>
       </c>
       <c r="C124" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D124" s="2">
-        <v>5000000</v>
+        <v>13850000</v>
       </c>
       <c r="E124" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F124" s="2">
-        <v>4112122</v>
+        <v>12550000</v>
       </c>
       <c r="G124" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.35">
@@ -3336,22 +3339,22 @@
         <v>45816</v>
       </c>
       <c r="B125" t="s">
+        <v>125</v>
+      </c>
+      <c r="C125" t="s">
         <v>124</v>
       </c>
-      <c r="C125" t="s">
-        <v>113</v>
-      </c>
       <c r="D125" s="2">
-        <v>13850000</v>
+        <v>1868500</v>
       </c>
       <c r="E125" t="s">
-        <v>117</v>
-      </c>
-      <c r="F125" s="2">
-        <v>12550000</v>
+        <v>112</v>
+      </c>
+      <c r="F125" t="s">
+        <v>114</v>
       </c>
       <c r="G125" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.35">
@@ -3362,19 +3365,19 @@
         <v>126</v>
       </c>
       <c r="C126" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D126" s="2">
-        <v>1868500</v>
+        <v>6110000</v>
       </c>
       <c r="E126" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F126" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G126" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.35">
@@ -3385,19 +3388,19 @@
         <v>127</v>
       </c>
       <c r="C127" t="s">
-        <v>125</v>
+        <v>113</v>
       </c>
       <c r="D127" s="2">
-        <v>6110000</v>
+        <v>1884900</v>
       </c>
       <c r="E127" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F127" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G127" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.35">
@@ -3408,19 +3411,19 @@
         <v>128</v>
       </c>
       <c r="C128" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D128" s="2">
-        <v>1884900</v>
+        <v>166400</v>
       </c>
       <c r="E128" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F128" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G128" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.35">
@@ -3428,22 +3431,22 @@
         <v>45816</v>
       </c>
       <c r="B129" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C129" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D129" s="2">
-        <v>166400</v>
+        <v>873600</v>
       </c>
       <c r="E129" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F129" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G129" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.35">
@@ -3451,39 +3454,39 @@
         <v>45816</v>
       </c>
       <c r="B130" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="C130" t="s">
-        <v>132</v>
+        <v>7</v>
       </c>
       <c r="D130" s="2">
-        <v>873600</v>
+        <v>760000</v>
       </c>
       <c r="E130" t="s">
-        <v>113</v>
-      </c>
-      <c r="F130" t="s">
-        <v>115</v>
-      </c>
-      <c r="G130" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A131" s="1">
-        <v>45816</v>
+        <v>45817</v>
       </c>
       <c r="B131" t="s">
-        <v>98</v>
+        <v>132</v>
       </c>
       <c r="C131" t="s">
-        <v>7</v>
+        <v>112</v>
       </c>
       <c r="D131" s="2">
-        <v>760000</v>
+        <v>360000</v>
       </c>
       <c r="E131" t="s">
-        <v>113</v>
+        <v>119</v>
+      </c>
+      <c r="F131" s="2">
+        <v>345011</v>
+      </c>
+      <c r="G131" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.35">
@@ -3494,19 +3497,19 @@
         <v>133</v>
       </c>
       <c r="C132" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D132" s="2">
-        <v>360000</v>
+        <v>3900000</v>
       </c>
       <c r="E132" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F132" s="2">
-        <v>345011</v>
+        <v>3417500</v>
       </c>
       <c r="G132" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.35">
@@ -3517,19 +3520,19 @@
         <v>134</v>
       </c>
       <c r="C133" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D133" s="2">
-        <v>3900000</v>
+        <v>560000</v>
       </c>
       <c r="E133" t="s">
-        <v>117</v>
-      </c>
-      <c r="F133" s="2">
-        <v>3417500</v>
+        <v>116</v>
+      </c>
+      <c r="F133" t="s">
+        <v>114</v>
       </c>
       <c r="G133" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.35">
@@ -3543,16 +3546,16 @@
         <v>113</v>
       </c>
       <c r="D134" s="2">
-        <v>560000</v>
+        <v>242400</v>
       </c>
       <c r="E134" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="F134" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G134" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.35">
@@ -3563,19 +3566,19 @@
         <v>136</v>
       </c>
       <c r="C135" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D135" s="2">
-        <v>242400</v>
+        <v>1832600</v>
       </c>
       <c r="E135" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F135" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G135" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.35">
@@ -3586,42 +3589,42 @@
         <v>137</v>
       </c>
       <c r="C136" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D136" s="2">
-        <v>1832600</v>
+        <v>748800</v>
       </c>
       <c r="E136" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F136" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G136" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A137" s="1">
-        <v>45817</v>
+        <v>45818</v>
       </c>
       <c r="B137" t="s">
         <v>138</v>
       </c>
       <c r="C137" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D137" s="2">
-        <v>748800</v>
+        <v>12756800</v>
       </c>
       <c r="E137" t="s">
         <v>113</v>
       </c>
       <c r="F137" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G137" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.35">
@@ -3632,19 +3635,19 @@
         <v>139</v>
       </c>
       <c r="C138" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D138" s="2">
-        <v>12756800</v>
+        <v>2087500</v>
       </c>
       <c r="E138" t="s">
-        <v>114</v>
-      </c>
-      <c r="F138" t="s">
-        <v>115</v>
+        <v>124</v>
+      </c>
+      <c r="F138" s="2">
+        <v>2080000</v>
       </c>
       <c r="G138" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.35">
@@ -3654,20 +3657,20 @@
       <c r="B139" t="s">
         <v>140</v>
       </c>
-      <c r="C139" t="s">
-        <v>113</v>
-      </c>
-      <c r="D139" s="2">
-        <v>2087500</v>
-      </c>
-      <c r="E139" t="s">
-        <v>125</v>
-      </c>
-      <c r="F139" s="2">
-        <v>2080000</v>
-      </c>
-      <c r="G139" t="s">
-        <v>117</v>
+      <c r="C139" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D139">
+        <v>13600300</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="F139">
+        <v>12934000</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.35">
@@ -3675,22 +3678,22 @@
         <v>45818</v>
       </c>
       <c r="B140" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D140">
-        <v>13600300</v>
+        <v>160000</v>
       </c>
       <c r="E140" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="F140">
-        <v>12934000</v>
+        <v>129</v>
+      </c>
+      <c r="F140" t="s">
+        <v>114</v>
       </c>
       <c r="G140" s="1" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.35">
@@ -3701,19 +3704,19 @@
         <v>143</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="D141">
-        <v>160000</v>
+        <v>1440000</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="F141" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G141" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.35">
@@ -3724,42 +3727,42 @@
         <v>144</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="D142">
-        <v>1440000</v>
+        <v>1840800</v>
       </c>
       <c r="E142" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F142" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G142" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A143" s="1">
-        <v>45818</v>
+        <v>45819</v>
       </c>
       <c r="B143" t="s">
         <v>145</v>
       </c>
-      <c r="C143" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="D143">
-        <v>1840800</v>
-      </c>
-      <c r="E143" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="F143" t="s">
-        <v>115</v>
-      </c>
-      <c r="G143" s="1" t="s">
-        <v>115</v>
+      <c r="C143" t="s">
+        <v>112</v>
+      </c>
+      <c r="D143" s="2">
+        <v>3167000</v>
+      </c>
+      <c r="E143" t="s">
+        <v>129</v>
+      </c>
+      <c r="F143" s="2">
+        <v>2861100</v>
+      </c>
+      <c r="G143" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.35">
@@ -3770,19 +3773,19 @@
         <v>146</v>
       </c>
       <c r="C144" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D144" s="2">
-        <v>3167000</v>
+        <v>9575555</v>
       </c>
       <c r="E144" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="F144" s="2">
-        <v>2861100</v>
+        <v>9564000</v>
       </c>
       <c r="G144" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.35">
@@ -3793,19 +3796,19 @@
         <v>147</v>
       </c>
       <c r="C145" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D145" s="2">
-        <v>9575555</v>
+        <v>2121323</v>
       </c>
       <c r="E145" t="s">
-        <v>125</v>
-      </c>
-      <c r="F145" s="2">
-        <v>9564000</v>
+        <v>120</v>
+      </c>
+      <c r="F145" t="s">
+        <v>114</v>
       </c>
       <c r="G145" t="s">
-        <v>130</v>
+        <v>114</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.35">
@@ -3816,19 +3819,19 @@
         <v>148</v>
       </c>
       <c r="C146" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D146" s="2">
-        <v>2121323</v>
+        <v>1477000</v>
       </c>
       <c r="E146" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="F146" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G146" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.35">
@@ -3842,16 +3845,16 @@
         <v>113</v>
       </c>
       <c r="D147" s="2">
-        <v>1477000</v>
+        <v>3161300</v>
       </c>
       <c r="E147" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="F147" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G147" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.35">
@@ -3862,19 +3865,19 @@
         <v>150</v>
       </c>
       <c r="C148" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D148" s="2">
-        <v>3161300</v>
+        <v>168000</v>
       </c>
       <c r="E148" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F148" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G148" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.35">
@@ -3885,19 +3888,19 @@
         <v>151</v>
       </c>
       <c r="C149" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D149" s="2">
-        <v>168000</v>
+        <v>3520000</v>
       </c>
       <c r="E149" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F149" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G149" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.35">
@@ -3905,22 +3908,22 @@
         <v>45819</v>
       </c>
       <c r="B150" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C150" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D150" s="2">
-        <v>3520000</v>
+        <v>1407600</v>
       </c>
       <c r="E150" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F150" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G150" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.35">
@@ -3928,22 +3931,22 @@
         <v>45819</v>
       </c>
       <c r="B151" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C151" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="D151" s="2">
-        <v>1407600</v>
+        <v>1500000</v>
       </c>
       <c r="E151" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="F151" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G151" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.35">
@@ -3951,22 +3954,22 @@
         <v>45819</v>
       </c>
       <c r="B152" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C152" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D152" s="2">
-        <v>1500000</v>
+        <v>3800000</v>
       </c>
       <c r="E152" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F152" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G152" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.35">
@@ -3974,45 +3977,45 @@
         <v>45819</v>
       </c>
       <c r="B153" t="s">
-        <v>155</v>
+        <v>133</v>
       </c>
       <c r="C153" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D153" s="2">
-        <v>3800000</v>
+        <v>4900000</v>
       </c>
       <c r="E153" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F153" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G153" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A154" s="1">
-        <v>45819</v>
+        <v>45820</v>
       </c>
       <c r="B154" t="s">
-        <v>134</v>
+        <v>155</v>
       </c>
       <c r="C154" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D154" s="2">
-        <v>4900000</v>
+        <v>6750000</v>
       </c>
       <c r="E154" t="s">
-        <v>132</v>
-      </c>
-      <c r="F154" t="s">
-        <v>115</v>
+        <v>119</v>
+      </c>
+      <c r="F154" s="2">
+        <v>6700000</v>
       </c>
       <c r="G154" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.35">
@@ -4023,19 +4026,19 @@
         <v>156</v>
       </c>
       <c r="C155" t="s">
+        <v>112</v>
+      </c>
+      <c r="D155" s="2">
+        <v>164000</v>
+      </c>
+      <c r="E155" t="s">
         <v>113</v>
       </c>
-      <c r="D155" s="2">
-        <v>6750000</v>
-      </c>
-      <c r="E155" t="s">
-        <v>120</v>
-      </c>
       <c r="F155" s="2">
-        <v>6700000</v>
+        <v>161000</v>
       </c>
       <c r="G155" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.35">
@@ -4046,19 +4049,19 @@
         <v>157</v>
       </c>
       <c r="C156" t="s">
+        <v>112</v>
+      </c>
+      <c r="D156" s="2">
+        <v>4710001</v>
+      </c>
+      <c r="E156" t="s">
+        <v>116</v>
+      </c>
+      <c r="F156" s="2">
+        <v>4679509</v>
+      </c>
+      <c r="G156" t="s">
         <v>113</v>
-      </c>
-      <c r="D156" s="2">
-        <v>164000</v>
-      </c>
-      <c r="E156" t="s">
-        <v>114</v>
-      </c>
-      <c r="F156" s="2">
-        <v>161000</v>
-      </c>
-      <c r="G156" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.35">
@@ -4066,19 +4069,19 @@
         <v>45820</v>
       </c>
       <c r="B157" t="s">
-        <v>158</v>
+        <v>121</v>
       </c>
       <c r="C157" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D157" s="2">
-        <v>4710001</v>
+        <v>280000</v>
       </c>
       <c r="E157" t="s">
-        <v>117</v>
-      </c>
-      <c r="F157" s="2">
-        <v>4679509</v>
+        <v>112</v>
+      </c>
+      <c r="F157" t="s">
+        <v>114</v>
       </c>
       <c r="G157" t="s">
         <v>114</v>
@@ -4089,22 +4092,22 @@
         <v>45820</v>
       </c>
       <c r="B158" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="C158" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D158" s="2">
-        <v>280000</v>
+        <v>2114600</v>
       </c>
       <c r="E158" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F158" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G158" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.35">
@@ -4112,22 +4115,22 @@
         <v>45820</v>
       </c>
       <c r="B159" t="s">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="C159" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D159" s="2">
-        <v>2114600</v>
+        <v>2069600</v>
       </c>
       <c r="E159" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F159" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G159" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.35">
@@ -4138,19 +4141,19 @@
         <v>159</v>
       </c>
       <c r="C160" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="D160" s="2">
-        <v>2069600</v>
+        <v>2667000</v>
       </c>
       <c r="E160" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F160" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G160" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.35">
@@ -4161,19 +4164,19 @@
         <v>160</v>
       </c>
       <c r="C161" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D161" s="2">
-        <v>2667000</v>
+        <v>1326000</v>
       </c>
       <c r="E161" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F161" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G161" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.35">
@@ -4184,19 +4187,19 @@
         <v>161</v>
       </c>
       <c r="C162" t="s">
-        <v>142</v>
+        <v>113</v>
       </c>
       <c r="D162" s="2">
-        <v>1326000</v>
+        <v>3450000</v>
       </c>
       <c r="E162" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F162" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G162" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.35">
@@ -4207,19 +4210,19 @@
         <v>162</v>
       </c>
       <c r="C163" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D163" s="2">
-        <v>3450000</v>
+        <v>2270000</v>
       </c>
       <c r="E163" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F163" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G163" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.35">
@@ -4227,22 +4230,22 @@
         <v>45820</v>
       </c>
       <c r="B164" t="s">
-        <v>163</v>
+        <v>142</v>
       </c>
       <c r="C164" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="D164" s="2">
-        <v>2270000</v>
+        <v>171700</v>
       </c>
       <c r="E164" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F164" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G164" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.35">
@@ -4250,22 +4253,22 @@
         <v>45820</v>
       </c>
       <c r="B165" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="C165" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D165" s="2">
-        <v>171700</v>
+        <v>808500</v>
       </c>
       <c r="E165" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F165" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G165" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.35">
@@ -4276,42 +4279,42 @@
         <v>164</v>
       </c>
       <c r="C166" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D166" s="2">
-        <v>808500</v>
+        <v>420000</v>
       </c>
       <c r="E166" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F166" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G166" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A167" s="1">
-        <v>45820</v>
+        <v>45821</v>
       </c>
       <c r="B167" t="s">
         <v>165</v>
       </c>
       <c r="C167" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D167" s="2">
-        <v>420000</v>
+        <v>5200510</v>
       </c>
       <c r="E167" t="s">
-        <v>113</v>
-      </c>
-      <c r="F167" t="s">
-        <v>115</v>
+        <v>116</v>
+      </c>
+      <c r="F167" s="2">
+        <v>5142422</v>
       </c>
       <c r="G167" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.35">
@@ -4322,19 +4325,19 @@
         <v>166</v>
       </c>
       <c r="C168" t="s">
+        <v>112</v>
+      </c>
+      <c r="D168" s="2">
+        <v>1545200</v>
+      </c>
+      <c r="E168" t="s">
+        <v>124</v>
+      </c>
+      <c r="F168" s="2">
+        <v>1541000</v>
+      </c>
+      <c r="G168" t="s">
         <v>113</v>
-      </c>
-      <c r="D168" s="2">
-        <v>5200510</v>
-      </c>
-      <c r="E168" t="s">
-        <v>117</v>
-      </c>
-      <c r="F168" s="2">
-        <v>5142422</v>
-      </c>
-      <c r="G168" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.35">
@@ -4345,16 +4348,16 @@
         <v>167</v>
       </c>
       <c r="C169" t="s">
+        <v>112</v>
+      </c>
+      <c r="D169" s="2">
+        <v>457700</v>
+      </c>
+      <c r="E169" t="s">
         <v>113</v>
       </c>
-      <c r="D169" s="2">
-        <v>1545200</v>
-      </c>
-      <c r="E169" t="s">
-        <v>125</v>
-      </c>
-      <c r="F169" s="2">
-        <v>1541000</v>
+      <c r="F169" t="s">
+        <v>114</v>
       </c>
       <c r="G169" t="s">
         <v>114</v>
@@ -4368,19 +4371,19 @@
         <v>168</v>
       </c>
       <c r="C170" t="s">
+        <v>112</v>
+      </c>
+      <c r="D170" s="2">
+        <v>470008</v>
+      </c>
+      <c r="E170" t="s">
         <v>113</v>
       </c>
-      <c r="D170" s="2">
-        <v>457700</v>
-      </c>
-      <c r="E170" t="s">
-        <v>114</v>
-      </c>
       <c r="F170" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G170" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.35">
@@ -4391,19 +4394,19 @@
         <v>169</v>
       </c>
       <c r="C171" t="s">
+        <v>112</v>
+      </c>
+      <c r="D171" s="2">
+        <v>1723555</v>
+      </c>
+      <c r="E171" t="s">
+        <v>120</v>
+      </c>
+      <c r="F171" s="2">
+        <v>1676000</v>
+      </c>
+      <c r="G171" t="s">
         <v>113</v>
-      </c>
-      <c r="D171" s="2">
-        <v>470008</v>
-      </c>
-      <c r="E171" t="s">
-        <v>114</v>
-      </c>
-      <c r="F171" t="s">
-        <v>115</v>
-      </c>
-      <c r="G171" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.35">
@@ -4414,16 +4417,16 @@
         <v>170</v>
       </c>
       <c r="C172" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D172" s="2">
-        <v>1723555</v>
+        <v>489600</v>
       </c>
       <c r="E172" t="s">
-        <v>121</v>
-      </c>
-      <c r="F172" s="2">
-        <v>1676000</v>
+        <v>112</v>
+      </c>
+      <c r="F172" t="s">
+        <v>114</v>
       </c>
       <c r="G172" t="s">
         <v>114</v>
@@ -4434,68 +4437,45 @@
         <v>45821</v>
       </c>
       <c r="B173" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="C173" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D173" s="2">
-        <v>489600</v>
+        <v>170000</v>
       </c>
       <c r="E173" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F173" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G173" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A174" s="1">
-        <v>43995</v>
+        <v>45821</v>
       </c>
       <c r="B174" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="C174" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D174" s="2">
-        <v>170000</v>
+        <v>3759500</v>
       </c>
       <c r="E174" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F174" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G174" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A175" s="1">
-        <v>43995</v>
-      </c>
-      <c r="B175" t="s">
-        <v>172</v>
-      </c>
-      <c r="C175" t="s">
-        <v>114</v>
-      </c>
-      <c r="D175" s="2">
-        <v>3759500</v>
-      </c>
-      <c r="E175" t="s">
-        <v>113</v>
-      </c>
-      <c r="F175" t="s">
-        <v>115</v>
-      </c>
-      <c r="G175" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -4504,8 +4484,8 @@
       <sortCondition ref="A1"/>
     </sortState>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G118">
-    <sortCondition descending="1" ref="A2:A118"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G117">
+    <sortCondition descending="1" ref="A2:A117"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>